<commit_message>
Rev.2 canonica: inferencia del Word alineada a Stata (Wald 0,33/0,717; Chow 15,55), do-file con Fisher n=80 y Bai-Perron de rp (2011Q2), hojas de trazabilidad del xlsx restauradas, validacion Python unica (corrida_canonica.py), manifiesto actualizado
</commit_message>
<xml_diff>
--- a/data/processed/base_cda.xlsx
+++ b/data/processed/base_cda.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="datos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="diccionario" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fuentes_trazabilidad" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7350,4 +7352,1198 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>variable</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fuente</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>regla_agregacion</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>anio</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Año calendario</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>trimestre</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Trimestre (1-4)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Etiqueta YYYYQn</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>i_Gs</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tasa efectiva CDA &lt;=365 días, bancos, moneda nacional (SERIE PRIMARIA)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BCP-SB, boletines 'Promedio de Tasas'</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>promedio de meses publicados del trimestre</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>84/84 (10 meses no publicados, ver fuentes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>i_USD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tasa efectiva CDA &lt;=365 días, bancos, moneda extranjera (SERIE PRIMARIA)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BCP-SB, 'Promedio de Tasas'</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>promedio de meses publicados</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>i_Gs_fdt</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CDA &lt;=365 Gs, último mes publicado del trimestre</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BCP-SB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>último mes publicado</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>i_USD_fdt</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CDA &lt;=365 USD, último mes publicado</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BCP-SB</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>último mes publicado</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>meses_cobertura</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cantidad de meses publicados usados en el promedio del trimestre</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BCP-SB</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>conteo</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ultimo_mes_publicado</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mes del dato fdt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BCP-SB</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tipo de cambio nominal Gs/USD, promedio del último mes del trimestre</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Gs/USD</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BCP, Anexo Estadístico, Cuadro 60a col E</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>valor del mes de cierre</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dolariz</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Participación de depósitos en moneda extranjera</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>% del total</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BCP, Anexo Estadístico, Cuadro 23a col O</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>valor del mes de cierre</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IPC_PY</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IPC Paraguay, nivel (dic-2017=100)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>índice</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BCP, Anexo Estadístico, Cuadro 15 col V</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>valor del mes de cierre</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>infl_PY_yoy</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Inflación interanual Paraguay (publicada)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BCP, Cuadro 15 col Y</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>valor del mes de cierre</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IPC_US</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CPI EEUU (CPIAUCSL), nivel</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>índice</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FRED</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>valor del mes de cierre</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>infl_US_yoy</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Inflación interanual EEUU</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>derivada de CPIAUCSL: (CPI_t/CPI_t-12 -1)x100</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>mes de cierre</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>FEDFUNDS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Federal Funds Effective Rate</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FRED</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>promedio de los 3 meses</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>i_Gs_vista</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tasa a la vista MN (referencia, NO CDA)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BCP, Cuadro 31 col C</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>promedio 3 meses</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>i_USD_vista</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Tasa a la vista ME (referencia, NO CDA)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BCP, Cuadro 31 Cont. col C</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>promedio 3 meses</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>84/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>i_Gs_pond</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CDA promedio ponderado MN (SENSIBILIDAD; empalme 2010/2011)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BCP: IF mensuales 2004-2010 + Cuadro 31 2011+</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>promedio 3 meses</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>83/84 (falta 2006Q4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>i_USD_pond</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CDA promedio ponderado ME (SENSIBILIDAD)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ídem</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>promedio 3 meses</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>83/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>i_Gs_fdt_pond</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ponderada MN, fin de trimestre</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ídem</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>último mes</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>83/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>i_USD_fdt_pond</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ponderada ME, fin de trimestre</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ídem</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>último mes</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>83/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>encaje_mn</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tasa de encaje legal MN, tramo &lt;=360 días (base)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Resoluciones BCP (docs/11_encaje_fuentes.md)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>vigente al cierre</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>49/84 (verificado 2012Q4+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>encaje_me</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Tasa de encaje legal ME, tramo &lt;=360 días (base)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Resoluciones BCP</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>vigente al cierre</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>49/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>encaje_mn_efec</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Encaje MN efectivo (incluye desencaje COVID 2020)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Resoluciones BCP</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>vigente al cierre</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>49/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>encaje_me_efec</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Encaje ME efectivo</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Resoluciones BCP</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>vigente al cierre</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>49/84</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tpm</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Tasa de Política Monetaria</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>% anual</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>BCP, TPM.xlsx oficial (data/raw/bcp/TPM.xlsx)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>promedio de meses del trimestre</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>55/84 (la TPM nace en may-2011; pre-2011 no existe, no es hueco)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>serie</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fuente_oficial_exacta</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>url_y_archivo_crudo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fecha_extraccion</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>reglas_y_notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>i_Gs / i_USD (y fdt)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BCP - Superintendencia de Bancos, boletines mensuales 'Promedio de Tasas', fila 'CERTIFIC. DEP. DE AHORRO' tramo '&lt;=365 dias', tasa efectiva, Bancos</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.bcp.gov.py (Promedio de Tasas; 242 boletines descargados en data/raw/bcp/promedio_tasas/full/)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Fuente única 2004-2024, sin empalme. 10 meses NO publicados por el BCP: 2005-07, 2006-03, 2006-11, 2006-12, 2007-01, 2007-05, 2007-07, 2013-04, 2013-05, 2014-04. Trimestre=promedio de meses publicados (meses_cobertura).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BCP - Anexo Estadístico del Informe Económico, Cuadro 60a, col E</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.bcp.gov.py/anexo-estadistico-del-informe-economico-i365 (archivo en data/raw/bcp/Anexo_Estadistico_Informe_Economico.xlsx)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Promedio mensual del mes de cierre del trimestre (la cotización diaria de cierre no existe homogénea 2004-2024).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dolariz</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BCP - Anexo Estadístico, Cuadro 23a, col O (depósitos sector privado, participación ME)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ídem Anexo</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mes de cierre. 2024Q2-Q4 marcados preliminares por la fuente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IPC_PY / infl_PY_yoy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BCP - Anexo Estadístico, Cuadro 15, cols V (índice) e Y (interanual publicada)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ídem Anexo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Mes de cierre; la inflación es la publicada por el BCP, no recalculada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IPC_US / infl_US_yoy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FRED, serie CPIAUCSL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=CPIAUCSL (data/raw/fred/CPIAUCSL.csv)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Nivel del mes de cierre; interanual derivada (CPI_t/CPI_t-12 -1)x100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FEDFUNDS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FRED, serie FEDFUNDS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=FEDFUNDS (data/raw/fred/FEDFUNDS.csv)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Promedio de los 3 meses del trimestre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>i_*_pond</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BCP: Informes de Indicadores Financieros mensuales 2004-2010 (PDF, data/raw/bcp/if_pdfs/ + _INVENTARIO.csv con URL por archivo) empalmados con Cuadro 31 del Anexo 2011-2024</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ver _INVENTARIO.csv y Anexo</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SOLO SENSIBILIDAD: empalme 2010/2011 (~0,7-0,8pp definicional) y composición de plazos variable. Hueco: 2006Q4 (PDF escaneado ilegible).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>encaje_*</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Resoluciones del BCP (Res. 30/2012 MN 18%, Res. 31/2012 ME 24%, tramo &lt;=360d; desencaje COVID 2020: MN 7 / ME 15)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>detalle y enlaces en docs/11_encaje_fuentes.md</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Cobertura verificada 2012Q4-2024Q4; 2004-2012Q3 vacío (resoluciones escaneadas pendientes de OCR). Salvedad de tramo: encaje corta en 360d, CDA en 365d.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tpm</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BCP - Tasa de Política Monetaria, archivo oficial TPM.xlsx (serie mensual desde may-2011)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.bcp.gov.py/web/institucional/tasa-de-politica-monetaria (data/raw/bcp/TPM.xlsx; mensual intermedio en data/processed/tpm_mensual.csv)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Trimestre = promedio de meses disponibles (2011Q2 = may+jun). Pre-2011: la TPM no existía (no es dato faltante).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>